<commit_message>
Publish Latest checklists 2026-11-01 (#1593)
Updates based on OWASP/wstg@0360cec
</commit_message>
<xml_diff>
--- a/checklists/checklist.xlsx
+++ b/checklists/checklist.xlsx
@@ -1548,7 +1548,7 @@
         </is>
       </c>
       <c r="C6" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/01-Information_Gathering/01-Conduct_Search_Engine_Reconnaissance_for_Information_Leakage", "Conduct Search Engine Reconnaissance for Information Leakage")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/01-Information_Gathering/01-Conduct_Search_Engine_Reconnaissance_for_Information_Leakage", "Conduct Search Engine Reconnaissance for Information Leakage")</f>
         <v/>
       </c>
       <c r="D6" s="16" t="inlineStr">
@@ -1571,7 +1571,7 @@
         </is>
       </c>
       <c r="C7" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/01-Information_Gathering/02-Fingerprint_Web_Server", "Fingerprint Web Server")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/01-Information_Gathering/02-Fingerprint_Web_Server", "Fingerprint Web Server")</f>
         <v/>
       </c>
       <c r="D7" s="16" t="inlineStr">
@@ -1594,7 +1594,7 @@
         </is>
       </c>
       <c r="C8" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/01-Information_Gathering/03-Review_Webserver_Metafiles_for_Information_Leakage", "Review Webserver Metafiles for Information Leakage")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/01-Information_Gathering/03-Review_Webserver_Metafiles_for_Information_Leakage", "Review Webserver Metafiles for Information Leakage")</f>
         <v/>
       </c>
       <c r="D8" s="16" t="inlineStr">
@@ -1618,7 +1618,7 @@
         </is>
       </c>
       <c r="C9" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/01-Information_Gathering/04-Attack_Surface_Identification", "Attack Surface Identification")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/01-Information_Gathering/04-Attack_Surface_Identification", "Attack Surface Identification")</f>
         <v/>
       </c>
       <c r="D9" s="16" t="inlineStr">
@@ -1644,7 +1644,7 @@
         </is>
       </c>
       <c r="C10" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/01-Information_Gathering/05-Review_Web_Page_Content_for_Information_Leakage", "Review Web Page Content for Information Leakage")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/01-Information_Gathering/05-Review_Web_Page_Content_for_Information_Leakage", "Review Web Page Content for Information Leakage")</f>
         <v/>
       </c>
       <c r="D10" s="16" t="inlineStr">
@@ -1669,7 +1669,7 @@
         </is>
       </c>
       <c r="C11" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/01-Information_Gathering/06-Identify_Application_Entry_Points", "Identify Application Entry Points")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/01-Information_Gathering/06-Identify_Application_Entry_Points", "Identify Application Entry Points")</f>
         <v/>
       </c>
       <c r="D11" s="16" t="inlineStr">
@@ -1692,7 +1692,7 @@
         </is>
       </c>
       <c r="C12" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/01-Information_Gathering/07-Map_Execution_Paths_Through_Application", "Map Execution Paths Through Application")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/01-Information_Gathering/07-Map_Execution_Paths_Through_Application", "Map Execution Paths Through Application")</f>
         <v/>
       </c>
       <c r="D12" s="16" t="inlineStr">
@@ -1715,7 +1715,7 @@
         </is>
       </c>
       <c r="C13" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/01-Information_Gathering/08-Fingerprint_Web_Application_Framework", "Fingerprint Web Application Framework")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/01-Information_Gathering/08-Fingerprint_Web_Application_Framework", "Fingerprint Web Application Framework")</f>
         <v/>
       </c>
       <c r="D13" s="16" t="inlineStr">
@@ -1738,7 +1738,7 @@
         </is>
       </c>
       <c r="C14" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/01-Information_Gathering/09-Fingerprint_Web_Application", "Fingerprint Web Application")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/01-Information_Gathering/09-Fingerprint_Web_Application", "Fingerprint Web Application")</f>
         <v/>
       </c>
       <c r="D14" s="16" t="inlineStr">
@@ -1761,7 +1761,7 @@
         </is>
       </c>
       <c r="C15" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/01-Information_Gathering/10-Map_Application_Architecture", "Map Application Architecture")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/01-Information_Gathering/10-Map_Application_Architecture", "Map Application Architecture")</f>
         <v/>
       </c>
       <c r="D15" s="16" t="inlineStr">
@@ -1820,7 +1820,7 @@
         </is>
       </c>
       <c r="C18" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/01-Network_Infrastructure_Configuration", "Network Infrastructure Configuration")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/01-Network_Infrastructure_Configuration", "Network Infrastructure Configuration")</f>
         <v/>
       </c>
       <c r="D18" s="16" t="inlineStr">
@@ -1845,7 +1845,7 @@
         </is>
       </c>
       <c r="C19" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/02-Application_Platform_Configuration", "Application Platform Configuration")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/02-Application_Platform_Configuration", "Application Platform Configuration")</f>
         <v/>
       </c>
       <c r="D19" s="16" t="inlineStr">
@@ -1871,7 +1871,7 @@
         </is>
       </c>
       <c r="C20" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/03-File_Extensions_Handling_for_Sensitive_Information", "File Extensions Handling for Sensitive Information")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/03-File_Extensions_Handling_for_Sensitive_Information", "File Extensions Handling for Sensitive Information")</f>
         <v/>
       </c>
       <c r="D20" s="16" t="inlineStr">
@@ -1894,7 +1894,7 @@
         </is>
       </c>
       <c r="C21" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/04-Review_Old_Backup_and_Unreferenced_Files_for_Sensitive_Information", "Review Old Backup and Unreferenced Files for Sensitive Information")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/04-Review_Old_Backup_and_Unreferenced_Files_for_Sensitive_Information", "Review Old Backup and Unreferenced Files for Sensitive Information")</f>
         <v/>
       </c>
       <c r="D21" s="16" t="inlineStr">
@@ -1918,7 +1918,7 @@
         </is>
       </c>
       <c r="C22" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/05-Enumerate_Infrastructure_and_Application_Admin_Interfaces", "Enumerate Infrastructure and Application Admin Interfaces")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/05-Enumerate_Infrastructure_and_Application_Admin_Interfaces", "Enumerate Infrastructure and Application Admin Interfaces")</f>
         <v/>
       </c>
       <c r="D22" s="16" t="inlineStr">
@@ -1942,7 +1942,7 @@
         </is>
       </c>
       <c r="C23" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/06-HTTP_Methods", "HTTP Methods")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/06-HTTP_Methods", "HTTP Methods")</f>
         <v/>
       </c>
       <c r="D23" s="16" t="inlineStr">
@@ -1967,7 +1967,7 @@
         </is>
       </c>
       <c r="C24" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/07-HTTP_Strict_Transport_Security", "HTTP Strict Transport Security")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/07-HTTP_Strict_Transport_Security", "HTTP Strict Transport Security")</f>
         <v/>
       </c>
       <c r="D24" s="16" t="inlineStr">
@@ -1992,7 +1992,7 @@
         </is>
       </c>
       <c r="C25" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/09-File_Permissions", "File Permissions")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/09-File_Permissions", "File Permissions")</f>
         <v/>
       </c>
       <c r="D25" s="16" t="inlineStr">
@@ -2017,7 +2017,7 @@
         </is>
       </c>
       <c r="C26" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/10-Subdomain_Takeover", "Subdomain Takeover")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/10-Subdomain_Takeover", "Subdomain Takeover")</f>
         <v/>
       </c>
       <c r="D26" s="16" t="inlineStr">
@@ -2042,7 +2042,7 @@
         </is>
       </c>
       <c r="C27" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/11-Cloud_Storage", "Cloud Storage")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/11-Cloud_Storage", "Cloud Storage")</f>
         <v/>
       </c>
       <c r="D27" s="16" t="inlineStr">
@@ -2067,7 +2067,7 @@
         </is>
       </c>
       <c r="C28" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/12-Content_Security_Policy", "Content Security Policy")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/12-Content_Security_Policy", "Content Security Policy")</f>
         <v/>
       </c>
       <c r="D28" s="16" t="inlineStr">
@@ -2090,7 +2090,7 @@
         </is>
       </c>
       <c r="C29" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/13-Path_Confusion", "Path Confusion")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/13-Path_Confusion", "Path Confusion")</f>
         <v/>
       </c>
       <c r="D29" s="16" t="inlineStr">
@@ -2114,7 +2114,7 @@
         </is>
       </c>
       <c r="C30" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/14-Other_HTTP_Security_Header_Misconfigurations", "Other HTTP Security Header Misconfigurations")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/14-Other_HTTP_Security_Header_Misconfigurations", "Other HTTP Security Header Misconfigurations")</f>
         <v/>
       </c>
       <c r="D30" s="16" t="inlineStr">
@@ -2139,7 +2139,7 @@
         </is>
       </c>
       <c r="C31" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/15-Feature_Flag_Security_Bypass", "Feature Flag Security Bypass")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/15-Feature_Flag_Security_Bypass", "Feature Flag Security Bypass")</f>
         <v/>
       </c>
       <c r="D31" s="16" t="inlineStr">
@@ -2202,7 +2202,7 @@
         </is>
       </c>
       <c r="C34" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management/01-Role_Definitions", "Role Definitions")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/03-Identity_Management/01-Role_Definitions", "Role Definitions")</f>
         <v/>
       </c>
       <c r="D34" s="16" t="inlineStr">
@@ -2227,7 +2227,7 @@
         </is>
       </c>
       <c r="C35" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management/02-User_Registration_Process", "User Registration Process")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/03-Identity_Management/02-User_Registration_Process", "User Registration Process")</f>
         <v/>
       </c>
       <c r="D35" s="16" t="inlineStr">
@@ -2251,7 +2251,7 @@
         </is>
       </c>
       <c r="C36" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management/03-Account_Provisioning_Process", "Account Provisioning Process")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/03-Identity_Management/03-Account_Provisioning_Process", "Account Provisioning Process")</f>
         <v/>
       </c>
       <c r="D36" s="16" t="inlineStr">
@@ -2274,7 +2274,7 @@
         </is>
       </c>
       <c r="C37" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management/04-Account_Enumeration_and_Guessable_User_Account", "Account Enumeration and Guessable User Account")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/03-Identity_Management/04-Account_Enumeration_and_Guessable_User_Account", "Account Enumeration and Guessable User Account")</f>
         <v/>
       </c>
       <c r="D37" s="16" t="inlineStr">
@@ -2298,7 +2298,7 @@
         </is>
       </c>
       <c r="C38" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management/05-Weak_or_Unenforced_Username_Policy", "Weak or Unenforced Username Policy")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/03-Identity_Management/05-Weak_or_Unenforced_Username_Policy", "Weak or Unenforced Username Policy")</f>
         <v/>
       </c>
       <c r="D38" s="16" t="inlineStr">
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="C41" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/01-Credentials_Transported_over_an_Encrypted_Channel", "Credentials Transported over an Encrypted Channel")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/04-Authentication/01-Credentials_Transported_over_an_Encrypted_Channel", "Credentials Transported over an Encrypted Channel")</f>
         <v/>
       </c>
       <c r="D41" s="16" t="inlineStr">
@@ -2380,7 +2380,7 @@
         </is>
       </c>
       <c r="C42" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/02-Default_Credentials", "Default Credentials")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/04-Authentication/02-Default_Credentials", "Default Credentials")</f>
         <v/>
       </c>
       <c r="D42" s="16" t="inlineStr">
@@ -2404,7 +2404,7 @@
         </is>
       </c>
       <c r="C43" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/03-Weak_Lock_Out_Mechanism", "Weak Lock Out Mechanism")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/04-Authentication/03-Weak_Lock_Out_Mechanism", "Weak Lock Out Mechanism")</f>
         <v/>
       </c>
       <c r="D43" s="16" t="inlineStr">
@@ -2428,7 +2428,7 @@
         </is>
       </c>
       <c r="C44" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/04-Bypassing_Authentication_Schema", "Bypassing Authentication Schema")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/04-Authentication/04-Bypassing_Authentication_Schema", "Bypassing Authentication Schema")</f>
         <v/>
       </c>
       <c r="D44" s="16" t="inlineStr">
@@ -2451,7 +2451,7 @@
         </is>
       </c>
       <c r="C45" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/05-Vulnerable_Remember_Password", "Vulnerable Remember Password")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/04-Authentication/05-Vulnerable_Remember_Password", "Vulnerable Remember Password")</f>
         <v/>
       </c>
       <c r="D45" s="16" t="inlineStr">
@@ -2474,7 +2474,7 @@
         </is>
       </c>
       <c r="C46" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/06-Browser_Cache_Weaknesses", "Browser Cache Weaknesses")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/04-Authentication/06-Browser_Cache_Weaknesses", "Browser Cache Weaknesses")</f>
         <v/>
       </c>
       <c r="D46" s="16" t="inlineStr">
@@ -2498,7 +2498,7 @@
         </is>
       </c>
       <c r="C47" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/07-Weak_Authentication_Methods", "Weak Authentication Methods")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/04-Authentication/07-Weak_Authentication_Methods", "Weak Authentication Methods")</f>
         <v/>
       </c>
       <c r="D47" s="16" t="inlineStr">
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="C48" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/08-Weak_Security_Question_Answer", "Weak Security Question Answer")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/04-Authentication/08-Weak_Security_Question_Answer", "Weak Security Question Answer")</f>
         <v/>
       </c>
       <c r="D48" s="16" t="inlineStr">
@@ -2545,7 +2545,7 @@
         </is>
       </c>
       <c r="C49" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/09-Weak_Password_Change_or_Reset_Functionalities", "Weak Password Change or Reset Functionalities")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/04-Authentication/09-Weak_Password_Change_or_Reset_Functionalities", "Weak Password Change or Reset Functionalities")</f>
         <v/>
       </c>
       <c r="D49" s="16" t="inlineStr">
@@ -2568,7 +2568,7 @@
         </is>
       </c>
       <c r="C50" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/10-Weaker_Authentication_in_Alternative_Channel", "Weaker Authentication in Alternative Channel")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/04-Authentication/10-Weaker_Authentication_in_Alternative_Channel", "Weaker Authentication in Alternative Channel")</f>
         <v/>
       </c>
       <c r="D50" s="16" t="inlineStr">
@@ -2592,7 +2592,7 @@
         </is>
       </c>
       <c r="C51" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/11-Multi-Factor_Authentication", "Multi-Factor Authentication (MFA)")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/04-Authentication/11-Multi-Factor_Authentication", "Multi-Factor Authentication (MFA)")</f>
         <v/>
       </c>
       <c r="D51" s="16" t="inlineStr">
@@ -2653,7 +2653,7 @@
         </is>
       </c>
       <c r="C54" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization/01-Directory_Traversal_File_Include", "Directory Traversal File Include")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/05-Authorization/01-Directory_Traversal_File_Include", "Directory Traversal File Include")</f>
         <v/>
       </c>
       <c r="D54" s="16" t="inlineStr">
@@ -2677,7 +2677,7 @@
         </is>
       </c>
       <c r="C55" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization/02-Bypassing_Authorization_Schema", "Bypassing Authorization Schema")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/05-Authorization/02-Bypassing_Authorization_Schema", "Bypassing Authorization Schema")</f>
         <v/>
       </c>
       <c r="D55" s="16" t="inlineStr">
@@ -2700,7 +2700,7 @@
         </is>
       </c>
       <c r="C56" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization/03-Privilege_Escalation", "Privilege Escalation")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/05-Authorization/03-Privilege_Escalation", "Privilege Escalation")</f>
         <v/>
       </c>
       <c r="D56" s="16" t="inlineStr">
@@ -2724,7 +2724,7 @@
         </is>
       </c>
       <c r="C57" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization/04-Insecure_Direct_Object_References", "Insecure Direct Object References")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/05-Authorization/04-Insecure_Direct_Object_References", "Insecure Direct Object References")</f>
         <v/>
       </c>
       <c r="D57" s="16" t="inlineStr">
@@ -2748,7 +2748,7 @@
         </is>
       </c>
       <c r="C58" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization/05-OAuth_Weaknesses", "OAuth Weaknesses")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/05-Authorization/05-OAuth_Weaknesses", "OAuth Weaknesses")</f>
         <v/>
       </c>
       <c r="D58" s="16" t="inlineStr">
@@ -2807,7 +2807,7 @@
         </is>
       </c>
       <c r="C61" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/01-Session_Management_Schema", "Session Management Schema")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/06-Session_Management/01-Session_Management_Schema", "Session Management Schema")</f>
         <v/>
       </c>
       <c r="D61" s="16" t="inlineStr">
@@ -2832,7 +2832,7 @@
         </is>
       </c>
       <c r="C62" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/02-Cookies_Attributes", "Cookies Attributes")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/06-Session_Management/02-Cookies_Attributes", "Cookies Attributes")</f>
         <v/>
       </c>
       <c r="D62" s="16" t="inlineStr">
@@ -2855,7 +2855,7 @@
         </is>
       </c>
       <c r="C63" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/03-Session_Fixation", "Session Fixation")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/06-Session_Management/03-Session_Fixation", "Session Fixation")</f>
         <v/>
       </c>
       <c r="D63" s="16" t="inlineStr">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="C64" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/04-Exposed_Session_Variables", "Exposed Session Variables")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/06-Session_Management/04-Exposed_Session_Variables", "Exposed Session Variables")</f>
         <v/>
       </c>
       <c r="D64" s="16" t="inlineStr">
@@ -2904,7 +2904,7 @@
         </is>
       </c>
       <c r="C65" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/05-Cross_Site_Request_Forgery", "Cross Site Request Forgery")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/06-Session_Management/05-Cross_Site_Request_Forgery", "Cross Site Request Forgery")</f>
         <v/>
       </c>
       <c r="D65" s="16" t="inlineStr">
@@ -2927,7 +2927,7 @@
         </is>
       </c>
       <c r="C66" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/06-Logout_Functionality", "Logout Functionality")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/06-Session_Management/06-Logout_Functionality", "Logout Functionality")</f>
         <v/>
       </c>
       <c r="D66" s="16" t="inlineStr">
@@ -2951,7 +2951,7 @@
         </is>
       </c>
       <c r="C67" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/07-Session_Timeout", "Session Timeout")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/06-Session_Management/07-Session_Timeout", "Session Timeout")</f>
         <v/>
       </c>
       <c r="D67" s="16" t="inlineStr">
@@ -2974,7 +2974,7 @@
         </is>
       </c>
       <c r="C68" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/08-Session_Puzzling", "Session Puzzling")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/06-Session_Management/08-Session_Puzzling", "Session Puzzling")</f>
         <v/>
       </c>
       <c r="D68" s="16" t="inlineStr">
@@ -2998,7 +2998,7 @@
         </is>
       </c>
       <c r="C69" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/09-Session_Hijacking", "Session Hijacking")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/06-Session_Management/09-Session_Hijacking", "Session Hijacking")</f>
         <v/>
       </c>
       <c r="D69" s="16" t="inlineStr">
@@ -3022,7 +3022,7 @@
         </is>
       </c>
       <c r="C70" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/10-JSON_Web_Tokens", "JSON Web Tokens")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/06-Session_Management/10-JSON_Web_Tokens", "JSON Web Tokens")</f>
         <v/>
       </c>
       <c r="D70" s="16" t="inlineStr">
@@ -3046,7 +3046,7 @@
         </is>
       </c>
       <c r="C71" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/11-Concurrent_Sessions", "Concurrent Sessions")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/06-Session_Management/11-Concurrent_Sessions", "Concurrent Sessions")</f>
         <v/>
       </c>
       <c r="D71" s="16" t="inlineStr">
@@ -3105,7 +3105,7 @@
         </is>
       </c>
       <c r="C74" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/01-Reflected_Cross_Site_Scripting", "Reflected Cross Site Scripting")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/07-Injection/01-Reflected_Cross_Site_Scripting", "Reflected Cross Site Scripting")</f>
         <v/>
       </c>
       <c r="D74" s="16" t="inlineStr">
@@ -3129,7 +3129,7 @@
         </is>
       </c>
       <c r="C75" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/02-Stored_Cross_Site_Scripting", "Stored Cross Site Scripting")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/07-Injection/02-Stored_Cross_Site_Scripting", "Stored Cross Site Scripting")</f>
         <v/>
       </c>
       <c r="D75" s="16" t="inlineStr">
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C76" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/03-HTTP_Verb_Tampering", "HTTP Verb Tampering")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/07-Injection/03-HTTP_Verb_Tampering", "HTTP Verb Tampering")</f>
         <v/>
       </c>
       <c r="D76" s="16" t="inlineStr">
@@ -3176,7 +3176,7 @@
         </is>
       </c>
       <c r="C77" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/04-HTTP_Parameter_Pollution", "HTTP Parameter Pollution")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/07-Injection/04-HTTP_Parameter_Pollution", "HTTP Parameter Pollution")</f>
         <v/>
       </c>
       <c r="D77" s="16" t="inlineStr">
@@ -3200,7 +3200,7 @@
         </is>
       </c>
       <c r="C78" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/05-SQL_Injection", "SQL Injection")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/07-Injection/05-SQL_Injection", "SQL Injection")</f>
         <v/>
       </c>
       <c r="D78" s="16" t="inlineStr">
@@ -3224,7 +3224,7 @@
         </is>
       </c>
       <c r="C79" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/06-LDAP_Injection", "LDAP Injection")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/07-Injection/06-LDAP_Injection", "LDAP Injection")</f>
         <v/>
       </c>
       <c r="D79" s="16" t="inlineStr">
@@ -3248,7 +3248,7 @@
         </is>
       </c>
       <c r="C80" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/07-XML_Injection", "XML Injection")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/07-Injection/07-XML_Injection", "XML Injection")</f>
         <v/>
       </c>
       <c r="D80" s="16" t="inlineStr">
@@ -3272,7 +3272,7 @@
         </is>
       </c>
       <c r="C81" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/08-SSI_Injection", "SSI Injection")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/07-Injection/08-SSI_Injection", "SSI Injection")</f>
         <v/>
       </c>
       <c r="D81" s="16" t="inlineStr">
@@ -3296,7 +3296,7 @@
         </is>
       </c>
       <c r="C82" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/09-XPath_Injection", "XPath Injection")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/07-Injection/09-XPath_Injection", "XPath Injection")</f>
         <v/>
       </c>
       <c r="D82" s="16" t="inlineStr">
@@ -3319,7 +3319,7 @@
         </is>
       </c>
       <c r="C83" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/10-IMAP_SMTP_Injection", "IMAP SMTP Injection")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/07-Injection/10-IMAP_SMTP_Injection", "IMAP SMTP Injection")</f>
         <v/>
       </c>
       <c r="D83" s="16" t="inlineStr">
@@ -3344,7 +3344,7 @@
         </is>
       </c>
       <c r="C84" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/11-Code_Injection", "Code Injection")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/07-Injection/11-Code_Injection", "Code Injection")</f>
         <v/>
       </c>
       <c r="D84" s="16" t="inlineStr">
@@ -3368,7 +3368,7 @@
         </is>
       </c>
       <c r="C85" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/12-Command_Injection", "Command Injection")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/07-Injection/12-Command_Injection", "Command Injection")</f>
         <v/>
       </c>
       <c r="D85" s="16" t="inlineStr">
@@ -3392,7 +3392,7 @@
         </is>
       </c>
       <c r="C86" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/13-Format_String_Injection", "Format String Injection")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/07-Injection/13-Format_String_Injection", "Format String Injection")</f>
         <v/>
       </c>
       <c r="D86" s="16" t="inlineStr">
@@ -3415,7 +3415,7 @@
         </is>
       </c>
       <c r="C87" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/14-Incubated_Vulnerability", "Incubated Vulnerability")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/07-Injection/14-Incubated_Vulnerability", "Incubated Vulnerability")</f>
         <v/>
       </c>
       <c r="D87" s="16" t="inlineStr">
@@ -3440,7 +3440,7 @@
         </is>
       </c>
       <c r="C88" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/15-HTTP_Response_Splitting", "HTTP Response Splitting")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/07-Injection/15-HTTP_Response_Splitting", "HTTP Response Splitting")</f>
         <v/>
       </c>
       <c r="D88" s="16" t="inlineStr">
@@ -3465,7 +3465,7 @@
         </is>
       </c>
       <c r="C89" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/16-HTTP_Request_Smuggling", "HTTP Request Smuggling")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/07-Injection/16-HTTP_Request_Smuggling", "HTTP Request Smuggling")</f>
         <v/>
       </c>
       <c r="D89" s="16" t="inlineStr">
@@ -3492,7 +3492,7 @@
         </is>
       </c>
       <c r="C90" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/17-Host_Header_Injection", "Host Header Injection")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/07-Injection/17-Host_Header_Injection", "Host Header Injection")</f>
         <v/>
       </c>
       <c r="D90" s="16" t="inlineStr">
@@ -3516,7 +3516,7 @@
         </is>
       </c>
       <c r="C91" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/18-Server-side_Template_Injection", "Server-side Template Injection")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/07-Injection/18-Server-side_Template_Injection", "Server-side Template Injection")</f>
         <v/>
       </c>
       <c r="D91" s="16" t="inlineStr">
@@ -3541,7 +3541,7 @@
         </is>
       </c>
       <c r="C92" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/19-Server-Side_Request_Forgery", "Server-Side Request Forgery")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/07-Injection/19-Server-Side_Request_Forgery", "Server-Side Request Forgery")</f>
         <v/>
       </c>
       <c r="D92" s="16" t="inlineStr">
@@ -3566,7 +3566,7 @@
         </is>
       </c>
       <c r="C93" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/20-Mass_Assignment", "Mass Assignment")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/07-Injection/20-Mass_Assignment", "Mass Assignment")</f>
         <v/>
       </c>
       <c r="D93" s="16" t="inlineStr">
@@ -3590,7 +3590,7 @@
         </is>
       </c>
       <c r="C94" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/21-CSV_Injection", "CSV Injection")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/07-Injection/21-CSV_Injection", "CSV Injection")</f>
         <v/>
       </c>
       <c r="D94" s="16" t="inlineStr">
@@ -3617,7 +3617,7 @@
         </is>
       </c>
       <c r="C95" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/22-Prototype_Pollution", "Prototype Pollution")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/07-Injection/22-Prototype_Pollution", "Prototype Pollution")</f>
         <v/>
       </c>
       <c r="D95" s="16" t="inlineStr">
@@ -3642,7 +3642,7 @@
         </is>
       </c>
       <c r="C96" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/23-Insecure_Deserialization", "Insecure Deserialization")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/07-Injection/23-Insecure_Deserialization", "Insecure Deserialization")</f>
         <v/>
       </c>
       <c r="D96" s="16" t="inlineStr">
@@ -3706,7 +3706,7 @@
         </is>
       </c>
       <c r="C99" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/08-Error_Handling/01-Improper_Error_Handling", "Improper Error Handling")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/08-Error_Handling/01-Improper_Error_Handling", "Improper Error Handling")</f>
         <v/>
       </c>
       <c r="D99" s="16" t="inlineStr">
@@ -3731,7 +3731,7 @@
         </is>
       </c>
       <c r="C100" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/08-Error_Handling/02-Stack_Traces", "Stack Traces")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/08-Error_Handling/02-Stack_Traces", "Stack Traces")</f>
         <v/>
       </c>
       <c r="D100" s="16" t="inlineStr">
@@ -3790,7 +3790,7 @@
         </is>
       </c>
       <c r="C103" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Weak_Cryptography/01-Weak_Transport_Layer_Security", "Weak Transport Layer Security")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/09-Weak_Cryptography/01-Weak_Transport_Layer_Security", "Weak Transport Layer Security")</f>
         <v/>
       </c>
       <c r="D103" s="16" t="inlineStr">
@@ -3815,7 +3815,7 @@
         </is>
       </c>
       <c r="C104" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Weak_Cryptography/02-Padding_Oracle", "Padding Oracle")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/09-Weak_Cryptography/02-Padding_Oracle", "Padding Oracle")</f>
         <v/>
       </c>
       <c r="D104" s="16" t="inlineStr">
@@ -3839,7 +3839,7 @@
         </is>
       </c>
       <c r="C105" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Weak_Cryptography/03-Sensitive_Information_Sent_via_Unencrypted_Channels", "Sensitive Information Sent via Unencrypted Channels")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/09-Weak_Cryptography/03-Sensitive_Information_Sent_via_Unencrypted_Channels", "Sensitive Information Sent via Unencrypted Channels")</f>
         <v/>
       </c>
       <c r="D105" s="16" t="inlineStr">
@@ -3863,7 +3863,7 @@
         </is>
       </c>
       <c r="C106" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Weak_Cryptography/04-Weak_Cryptographic_Primitives", "Weak Cryptographic Primitives")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/09-Weak_Cryptography/04-Weak_Cryptographic_Primitives", "Weak Cryptographic Primitives")</f>
         <v/>
       </c>
       <c r="D106" s="16" t="inlineStr">
@@ -3922,7 +3922,7 @@
         </is>
       </c>
       <c r="C109" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/01-Business_Logic_Data_Validation", "Business Logic Data Validation")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/10-Business_Logic/01-Business_Logic_Data_Validation", "Business Logic Data Validation")</f>
         <v/>
       </c>
       <c r="D109" s="16" t="inlineStr">
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C110" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/02-Ability_to_Forge_Requests", "Ability to Forge Requests")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/10-Business_Logic/02-Ability_to_Forge_Requests", "Ability to Forge Requests")</f>
         <v/>
       </c>
       <c r="D110" s="16" t="inlineStr">
@@ -3972,7 +3972,7 @@
         </is>
       </c>
       <c r="C111" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/03-Integrity_Checks", "Integrity Checks")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/10-Business_Logic/03-Integrity_Checks", "Integrity Checks")</f>
         <v/>
       </c>
       <c r="D111" s="16" t="inlineStr">
@@ -3998,7 +3998,7 @@
         </is>
       </c>
       <c r="C112" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/04-Process_Timing", "Process Timing")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/10-Business_Logic/04-Process_Timing", "Process Timing")</f>
         <v/>
       </c>
       <c r="D112" s="16" t="inlineStr">
@@ -4022,7 +4022,7 @@
         </is>
       </c>
       <c r="C113" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/05-Number_of_Times_a_Function_Can_Be_Used_Limits", "Number of Times a Function Can Be Used Limits")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/10-Business_Logic/05-Number_of_Times_a_Function_Can_Be_Used_Limits", "Number of Times a Function Can Be Used Limits")</f>
         <v/>
       </c>
       <c r="D113" s="16" t="inlineStr">
@@ -4046,7 +4046,7 @@
         </is>
       </c>
       <c r="C114" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/06-Circumvention_of_Work_Flows", "Circumvention of Work Flows")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/10-Business_Logic/06-Circumvention_of_Work_Flows", "Circumvention of Work Flows")</f>
         <v/>
       </c>
       <c r="D114" s="16" t="inlineStr">
@@ -4070,7 +4070,7 @@
         </is>
       </c>
       <c r="C115" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/07-Defenses_Against_Application_Misuse", "Defenses Against Application Misuse")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/10-Business_Logic/07-Defenses_Against_Application_Misuse", "Defenses Against Application Misuse")</f>
         <v/>
       </c>
       <c r="D115" s="16" t="inlineStr">
@@ -4095,7 +4095,7 @@
         </is>
       </c>
       <c r="C116" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/08-Upload_of_Unexpected_File_Types", "Upload of Unexpected File Types")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/10-Business_Logic/08-Upload_of_Unexpected_File_Types", "Upload of Unexpected File Types")</f>
         <v/>
       </c>
       <c r="D116" s="16" t="inlineStr">
@@ -4120,7 +4120,7 @@
         </is>
       </c>
       <c r="C117" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/09-Upload_of_Malicious_Files", "Upload of Malicious Files")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/10-Business_Logic/09-Upload_of_Malicious_Files", "Upload of Malicious Files")</f>
         <v/>
       </c>
       <c r="D117" s="16" t="inlineStr">
@@ -4148,7 +4148,7 @@
         </is>
       </c>
       <c r="C118" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/10-Payment_Functionality", "Payment Functionality")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/10-Business_Logic/10-Payment_Functionality", "Payment Functionality")</f>
         <v/>
       </c>
       <c r="D118" s="16" t="inlineStr">
@@ -4209,7 +4209,7 @@
         </is>
       </c>
       <c r="C121" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/01-DOM-based_Cross_Site_Scripting", "DOM-Based Cross Site Scripting")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/11-Client-side/01-DOM-based_Cross_Site_Scripting", "DOM-Based Cross Site Scripting")</f>
         <v/>
       </c>
       <c r="D121" s="16" t="inlineStr">
@@ -4233,7 +4233,7 @@
         </is>
       </c>
       <c r="C122" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/02-JavaScript_Execution", "JavaScript Execution")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/11-Client-side/02-JavaScript_Execution", "JavaScript Execution")</f>
         <v/>
       </c>
       <c r="D122" s="16" t="inlineStr">
@@ -4256,7 +4256,7 @@
         </is>
       </c>
       <c r="C123" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/03-HTML_Injection", "HTML Injection")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/11-Client-side/03-HTML_Injection", "HTML Injection")</f>
         <v/>
       </c>
       <c r="D123" s="16" t="inlineStr">
@@ -4279,7 +4279,7 @@
         </is>
       </c>
       <c r="C124" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/04-Client-side_URL_Redirect", "Client-side URL Redirect")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/11-Client-side/04-Client-side_URL_Redirect", "Client-side URL Redirect")</f>
         <v/>
       </c>
       <c r="D124" s="16" t="inlineStr">
@@ -4303,7 +4303,7 @@
         </is>
       </c>
       <c r="C125" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/05-CSS_Injection", "CSS Injection")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/11-Client-side/05-CSS_Injection", "CSS Injection")</f>
         <v/>
       </c>
       <c r="D125" s="16" t="inlineStr">
@@ -4327,7 +4327,7 @@
         </is>
       </c>
       <c r="C126" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/06-Client-side_Resource_Manipulation", "Client-side Resource Manipulation")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/11-Client-side/06-Client-side_Resource_Manipulation", "Client-side Resource Manipulation")</f>
         <v/>
       </c>
       <c r="D126" s="16" t="inlineStr">
@@ -4351,7 +4351,7 @@
         </is>
       </c>
       <c r="C127" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/07-Cross_Origin_Resource_Sharing", "Cross Origin Resource Sharing")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/11-Client-side/07-Cross_Origin_Resource_Sharing", "Cross Origin Resource Sharing")</f>
         <v/>
       </c>
       <c r="D127" s="16" t="inlineStr">
@@ -4375,7 +4375,7 @@
         </is>
       </c>
       <c r="C128" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/09-Clickjacking", "Clickjacking")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/11-Client-side/09-Clickjacking", "Clickjacking")</f>
         <v/>
       </c>
       <c r="D128" s="16" t="inlineStr">
@@ -4398,7 +4398,7 @@
         </is>
       </c>
       <c r="C129" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/10-WebSockets", "WebSockets")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/11-Client-side/10-WebSockets", "WebSockets")</f>
         <v/>
       </c>
       <c r="D129" s="16" t="inlineStr">
@@ -4422,7 +4422,7 @@
         </is>
       </c>
       <c r="C130" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/11-Web_Messaging", "Web Messaging")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/11-Client-side/11-Web_Messaging", "Web Messaging")</f>
         <v/>
       </c>
       <c r="D130" s="16" t="inlineStr">
@@ -4446,7 +4446,7 @@
         </is>
       </c>
       <c r="C131" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/12-Browser_Storage", "Browser Storage")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/11-Client-side/12-Browser_Storage", "Browser Storage")</f>
         <v/>
       </c>
       <c r="D131" s="16" t="inlineStr">
@@ -4470,7 +4470,7 @@
         </is>
       </c>
       <c r="C132" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/13-Cross_Site_Script_Inclusion", "Cross Site Script Inclusion")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/11-Client-side/13-Cross_Site_Script_Inclusion", "Cross Site Script Inclusion")</f>
         <v/>
       </c>
       <c r="D132" s="16" t="inlineStr">
@@ -4494,7 +4494,7 @@
         </is>
       </c>
       <c r="C133" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/14-Reverse_Tabnabbing", "Reverse Tabnabbing")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/11-Client-side/14-Reverse_Tabnabbing", "Reverse Tabnabbing")</f>
         <v/>
       </c>
       <c r="D133" s="16" t="inlineStr">
@@ -4517,7 +4517,7 @@
         </is>
       </c>
       <c r="C134" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/15-Client-Side_Template_Injection", "Client-side Template Injection")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/11-Client-side/15-Client-Side_Template_Injection", "Client-side Template Injection")</f>
         <v/>
       </c>
       <c r="D134" s="16" t="inlineStr">
@@ -4578,7 +4578,7 @@
         </is>
       </c>
       <c r="C137" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/01-API_Reconnaissance", "API Reconnaissance")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/12-API_Testing/01-API_Reconnaissance", "API Reconnaissance")</f>
         <v/>
       </c>
       <c r="D137" s="16" t="inlineStr">
@@ -4603,7 +4603,7 @@
         </is>
       </c>
       <c r="C138" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/02-API_Broken_Object_Level_Authorization", "API Broken Object Level Authorization")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/12-API_Testing/02-API_Broken_Object_Level_Authorization", "API Broken Object Level Authorization")</f>
         <v/>
       </c>
       <c r="D138" s="16" t="inlineStr">
@@ -4626,7 +4626,7 @@
         </is>
       </c>
       <c r="C139" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/03-Excessive_Data_Exposure", "Excessive Data Exposure")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/12-API_Testing/03-Excessive_Data_Exposure", "Excessive Data Exposure")</f>
         <v/>
       </c>
       <c r="D139" s="16" t="inlineStr">
@@ -4651,7 +4651,7 @@
         </is>
       </c>
       <c r="C140" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/04-API_Broken_Function_Level_Authorization", "API Broken Function Level Authorization")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/12-API_Testing/04-API_Broken_Function_Level_Authorization", "API Broken Function Level Authorization")</f>
         <v/>
       </c>
       <c r="D140" s="16" t="inlineStr">
@@ -4674,7 +4674,7 @@
         </is>
       </c>
       <c r="C141" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/99-GraphQL", "GraphQL")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/12-API_Testing/99-GraphQL", "GraphQL")</f>
         <v/>
       </c>
       <c r="D141" s="16" t="inlineStr">
@@ -4735,7 +4735,7 @@
         </is>
       </c>
       <c r="C144" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/13-WebAssembly_Testing/01-WebAssembly_Reconnaissance", "WebAssembly Reconnaissance")</f>
+        <f>HYPERLINK("https://wstg.owasp.org/latest/4-Web_Application_Security_Testing/13-WebAssembly_Testing/01-WebAssembly_Reconnaissance", "WebAssembly Reconnaissance")</f>
         <v/>
       </c>
       <c r="D144" s="16" t="inlineStr">

</xml_diff>